<commit_message>
Add completed DeepWeeds GPU results
</commit_message>
<xml_diff>
--- a/submissions/2A202602415_nguyen_hong_cuong/results.xlsx
+++ b/submissions/2A202602415_nguyen_hong_cuong/results.xlsx
@@ -17,12 +17,12 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$N$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$K$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$M$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PerClass'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Latency'!$A$1:$M$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PerClass'!$A$1:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Latency'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$M$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -30,7 +30,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -69,12 +71,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -446,18 +451,18 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="19" customWidth="1" min="12" max="12"/>
-    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -504,22 +509,22 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>best_epoch</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>macro_F1_val</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>top1_val</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>train_s_per_epoch</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>latency_batch1_ms</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
@@ -536,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -544,226 +549,322 @@
           <t>resnet50</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ImageNet-1K</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>23.526473</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>4.087154688</v>
+      </c>
       <c r="F2" s="2" t="n">
         <v>224</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.7944939086397085</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.852042273636104</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>44.92886075700005</v>
+      </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Awaiting real GPU log</t>
+          <t>Full fold-0 Colab T4 run</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>resnext50_32x4d</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ImageNet-1K</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>23.526473</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>4.087154688</v>
+      </c>
       <c r="F3" s="2" t="n">
         <v>224</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.8061377620888833</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>0.8586118251928021</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>45.65146268060007</v>
+      </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Awaiting real GPU log</t>
+          <t>Full fold-0 Colab T4 run</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ImageNet-1K</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>23.526473</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>4.087154688</v>
+      </c>
       <c r="F4" s="2" t="n">
         <v>224</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.7937857616510409</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0.8500428449014568</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>46.02826896010001</v>
+      </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Awaiting real GPU log</t>
+          <t>Full fold-0 Colab T4 run</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>deit_small_patch16_224</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>ImageNet-1K</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>4.454770176</v>
+      </c>
       <c r="F5" s="2" t="n">
         <v>224</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0.9657669811987409</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>0.9728648957440731</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>57.99184297240022</v>
+      </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Awaiting real GPU log</t>
+          <t>Full fold-0 Colab T4 run</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>B05</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>swin_tiny_patch4_window7_224</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ImageNet-1K</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>4.454770176</v>
+      </c>
       <c r="F6" s="2" t="n">
         <v>224</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0.9613178589936867</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0.967723507569266</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>57.71141547600018</v>
+      </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Awaiting real GPU log</t>
+          <t>Full fold-0 Colab T4 run</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>B06</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>efficientnet_b0</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ImageNet-1K</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>4.454770176</v>
+      </c>
       <c r="F7" s="2" t="n">
         <v>224</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0.9648626469387582</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>0.9725792630676949</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>58.1627025658001</v>
+      </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Awaiting real GPU log</t>
+          <t>Full fold-0 Colab T4 run</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N7"/>
-  <conditionalFormatting sqref="I2:I500">
+  <conditionalFormatting sqref="J2:J7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -775,7 +876,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J500">
+  <conditionalFormatting sqref="K2:K7">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -797,20 +898,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -826,45 +926,40 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>axis_A_to_G</t>
+          <t>recipe</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>difference_from_T00</t>
+          <t>seed</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>macro_F1_val</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>macro_F1_val</t>
+          <t>top1_val</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>top1_val</t>
+          <t>delta_vs_T00_seed</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>delta_vs_T00</t>
+          <t>best_epoch</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>rare_class_F1</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -878,430 +973,253 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>select from validation</t>
+          <t>resnet50</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>baseline recipe</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
+          <t>ImageNet pretrained; basic augmentation; CE; no mixing; no EMA</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>0.7944939086397085</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.852042273636104</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Locked from validation</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>select from validation</t>
+          <t>resnet50</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>init=scratch</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
+          <t>ImageNet pretrained; basic augmentation; CE; no mixing; no EMA</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.8061377620888833</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.8586118251928021</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Locked from validation</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>select from validation</t>
+          <t>resnet50</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>init=frozen</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n">
+          <t>ImageNet pretrained; basic augmentation; CE; no mixing; no EMA</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.7937857616510409</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.8500428449014568</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Locked from validation</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>select from validation</t>
+          <t>convnext_tiny</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>aug=color</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
+          <t>ImageNet pretrained; RandAugment; weighted CE; CutMix; EMA</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>0.9657669811987409</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.9728648957440731</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.1712730725590325</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Locked from validation</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>select from validation</t>
+          <t>convnext_tiny</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>aug=randaug</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
+          <t>ImageNet pretrained; RandAugment; weighted CE; CutMix; EMA</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.9613178589936867</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.967723507569266</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.1551800969048034</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Locked from validation</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>select from validation</t>
+          <t>convnext_tiny</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>loss=label_smoothing(0.1)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>ImageNet pretrained; RandAugment; weighted CE; CutMix; EMA</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.9648626469387582</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.9725792630676949</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.1710768852877174</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Locked from validation</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>T06</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>select from validation</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>loss=focal(gamma=2)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>T07</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>select from validation</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>loss=class_weighted(beta=0.9999)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>T08</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>select from validation</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>mixup(alpha=0.4)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>T09</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>select from validation</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>cutmix(alpha=1.0)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>T10</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>select from validation</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>EMA(decay=0.999)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>One-factor comparison</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K12"/>
-  <conditionalFormatting sqref="F2:F500">
+  <autoFilter ref="A1:J7"/>
+  <conditionalFormatting sqref="E2:E7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1313,20 +1231,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G500">
+  <conditionalFormatting sqref="F2:F7">
     <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="00FEE2E2"/>
-        <color rgb="00FEF3C7"/>
-        <color rgb="00DCFCE7"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I500">
-    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1347,22 +1253,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1378,55 +1281,40 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>model_checkpoint</t>
+          <t>configuration</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>seed</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>views</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>macro_F1_val</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>top1_val</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>ECE_val</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>p50_ms_batch1</t>
+          <t>latency_batch1_ms</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>p95_ms_batch1</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>p99_ms_batch1</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>images_per_s</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>relative_cost_vs_I00</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1440,232 +1328,241 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>one view</t>
+          <t>one view FP32</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>best validation checkpoint</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="F2" s="3" t="n">
+        <v>0.7944939086397085</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.852042273636104</v>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy measured; batch-1 latency was not benchmarked</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_ACCURACY</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>I01</t>
+          <t>I00</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>horizontal flip TTA</t>
+          <t>one view FP32</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>best validation checkpoint</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.8061377620888833</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.8586118251928021</v>
+      </c>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy measured; batch-1 latency was not benchmarked</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_ACCURACY</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>I02</t>
+          <t>I00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>five crop TTA</t>
+          <t>one view FP32</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>best validation checkpoint</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.7937857616510409</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.8500428449014568</v>
+      </c>
       <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy measured; batch-1 latency was not benchmarked</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_ACCURACY</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>I03</t>
+          <t>I00</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>logit/probability aggregation</t>
+          <t>one view FP32</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>best validation checkpoint</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.9657669811987409</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.9728648957440731</v>
+      </c>
       <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy measured; batch-1 latency was not benchmarked</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_ACCURACY</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>I04</t>
+          <t>I00</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>temperature scaling fitted on val</t>
+          <t>one view FP32</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>best validation checkpoint</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.9613178589936867</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.967723507569266</v>
+      </c>
       <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy measured; batch-1 latency was not benchmarked</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_ACCURACY</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>I05</t>
+          <t>I00</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>probability ensemble</t>
+          <t>one view FP32</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>best validation checkpoint</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.9648626469387582</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.9725792630676949</v>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>I06</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Conv-BN fusion or FP16</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>best validation checkpoint</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy measured; batch-1 latency was not benchmarked</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_ACCURACY</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M8"/>
-  <conditionalFormatting sqref="E2:E500">
+  <autoFilter ref="A1:J7"/>
+  <conditionalFormatting sqref="F2:F7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1677,7 +1574,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F500">
+  <conditionalFormatting sqref="G2:G7">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1699,17 +1596,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
@@ -1757,7 +1654,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>mean_plus_minus_std</t>
+          <t>NLL_test</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -1766,9 +1663,237 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>resnet50 + I00</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.7944939086397085</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.7929493211847001</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.8477331052181352</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.7502110052098087</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.02985996620758479</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.4443433538237051</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>resnet50 + I00</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.8061377620888833</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.8095467521835746</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.861134873110921</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.7774973562218364</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.02374400996293137</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.415932874272281</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>resnet50 + I00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.7937857616510409</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.7938730820193965</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.850014257199886</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.7542708991217382</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.02452597955802679</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.4495061206865504</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>convnext_tiny + I00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.9657669811987409</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.9669165092737804</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.9726261762189906</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.9790335373532122</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.02438358489307115</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0.1140593185447561</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>convnext_tiny + I00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.9613178589936867</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.9618479610235874</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.9680638722554891</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.9752962148108062</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.02449096795551749</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0.1219636217634922</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>convnext_tiny + I00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.9648626469387582</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.9677437912752774</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.9729113202167095</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.9762717566392369</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.02412740816652403</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0.1122421569398458</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
-  <conditionalFormatting sqref="D2:D500">
+  <autoFilter ref="A1:J7"/>
+  <conditionalFormatting sqref="D2:D7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1780,7 +1905,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E500">
+  <conditionalFormatting sqref="E2:E7">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1792,8 +1917,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F500">
+  <conditionalFormatting sqref="F2:F7">
     <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00FEE2E2"/>
+        <color rgb="00FEF3C7"/>
+        <color rgb="00DCFCE7"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G7">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1814,16 +1951,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1844,29 +1984,740 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>precision</t>
+          <t>precision_mean</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>recall</t>
+          <t>precision_std</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>recall_mean</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>recall_std</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>F1_mean</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>F1_std</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Chinee apple</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.9189639129223474</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.01028386600552355</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.4675516224188791</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.03139203046282118</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.6193294606271776</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.02756163352703808</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>213</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.8751456887465622</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.009515731971982322</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.810641627543036</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.02218692782278216</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.84150200121162</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.01063018240773423</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>207</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.8904845450475474</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.0272124785847693</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.9339774557165862</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.01952392214650912</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.9113236287488805</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.006955326407164429</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>205</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.9190000307021583</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.01987591166013818</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.6373983739837398</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.03661245609495191</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.7519993294492545</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0.0199364810373803</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Prickly acacia</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>213</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.7802709899749374</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.01282232568697496</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.7464788732394365</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.0487901635934895</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.7626860970748571</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0.03184865835737994</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Rubber vine</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>202</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.9167308225365232</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.01163711159205356</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.7425742574257427</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.026195557535293</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.8202635012175185</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0.01407928277123361</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Siam weed</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.8776959656389017</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.009944470502913026</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.8558139534883721</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.009302325581395321</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.8665625813166797</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0.004684708047033127</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Snake weed</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>204</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.7414110731287797</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.02771181347512866</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0.687908496732026</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0.03263886332587937</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0.7128126932640969</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0.005950175237147006</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1822</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.8490124660960916</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.01452144921884767</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.9635931211123308</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.001764297614524836</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.9026281732529293</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0.007429078556815334</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Chinee apple</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.9638778147109232</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.01151560476972963</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>0.9424778761061946</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0.008849557522123908</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>0.9530285990688675</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>0.007970134341528714</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Lantana</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>213</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.9414659468438539</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.01860218294243846</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.9765258215962441</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.00469483568075113</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0.9585855129493787</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.007877744753023542</v>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Parkinsonia</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>207</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.9716500114139305</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.009076509959669413</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0.9903381642512077</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0.004830917874396101</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0.980872033976865</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.00225512052464292</v>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Parthenium</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>205</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.9774009974516517</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.01001319885492861</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.983739837398374</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.007451342593424136</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.9805589020385987</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.008733328440716876</v>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Prickly acacia</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>213</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0.9065602139050797</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0.01302732151240655</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0.9859154929577465</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0.004694835680751186</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0.9445582993459544</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.009107558065593064</v>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Rubber vine</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>202</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.9677281699133874</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0.005203032380102386</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.9884488448844885</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.007562006097286872</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0.9779546015906152</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.002514599838993388</v>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Siam weed</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>215</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0.9414529882366249</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0.01424408671901348</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>0.9937984496124032</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0.00537070017850813</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0.966852604791112</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0.005369687720396111</v>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Snake weed</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>204</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.9322663467543881</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0.008853885516836919</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.9656862745098039</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.008490445135141526</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0.9486384307301269</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.003603342574106219</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>1822</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.9924806121983724</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0.002502592312722057</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0.9648737650933041</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0.004689354415651729</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0.9784758002264172</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0.002152865961513105</v>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED_3_SEEDS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
-  <conditionalFormatting sqref="F2:F500">
+  <autoFilter ref="A1:J19"/>
+  <conditionalFormatting sqref="H2:H19">
     <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00FEE2E2"/>
+        <color rgb="00FEF3C7"/>
+        <color rgb="00DCFCE7"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I19">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1887,22 +2738,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1933,47 +2782,115 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>BN_fused</t>
+          <t>mean_train_epoch_s</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>p50_ms</t>
+          <t>p50_inference_ms</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>p95_ms</t>
+          <t>p95_inference_ms</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>p99_ms</t>
+          <t>p99_inference_ms</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>images_per_s</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>warmup</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>iterations</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
           <t>status</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA T4</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>AMP training / FP32 export</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>224</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>45.53619746590005</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Training time measured; inference latency not measured</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA T4</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>AMP training / FP32 export</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>224</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>57.95532033806683</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Training time measured; inference latency not measured</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M1"/>
+  <autoFilter ref="A1:K3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1984,19 +2901,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2017,95 +2937,156 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>macro_F1_val</t>
+          <t>macro_F1_val_mean</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>top1_val</t>
+          <t>macro_F1_test_mean</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>macro_F1_test_std</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>top1_test_mean</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>balanced_acc_test_mean</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ECE_test_mean</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>params_M</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>p95_ms_batch1</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>relative_cost</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>GMAC</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>evidence_note</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>No experiment metrics are populated until real GPU runs finish.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Select only from validation; test once per final seed.</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+          <t>convnext_tiny: ImageNet pretrained; RandAugment; weighted CE; CutMix; EMA</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.9639824957103954</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.9655027538575484</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.0031920576235212</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.9712004562303963</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.9768671696010851</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.02433398700503756</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>4.454770176</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>eval.py over three independent seeds</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EDA</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Fold 0 split verification</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>train=10501, val=3501, test=3507; disjoint; union=17509</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
+          <t>resnet50: ImageNet pretrained; basic augmentation; CE; no mixing; no EMA</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.7981391441265441</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.7987897184625571</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.009327307455866419</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.852960745176314</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.7606597535177944</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.02604331857618098</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>23.526473</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>4.087154688</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>eval.py over three independent seeds</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J3"/>
-  <conditionalFormatting sqref="D2:D500">
+  <autoFilter ref="A1:M3"/>
+  <conditionalFormatting sqref="D2:D3">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -2117,8 +3098,44 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E500">
+  <conditionalFormatting sqref="E2:E3">
     <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00FEE2E2"/>
+        <color rgb="00FEF3C7"/>
+        <color rgb="00DCFCE7"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F3">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00FEE2E2"/>
+        <color rgb="00FEF3C7"/>
+        <color rgb="00DCFCE7"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G3">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00FEE2E2"/>
+        <color rgb="00FEF3C7"/>
+        <color rgb="00DCFCE7"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H3">
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>